<commit_message>
Accepted the BOM updates
</commit_message>
<xml_diff>
--- a/EQs/EQ UCT Sonar PCB Manufacture_BOM .xlsx
+++ b/EQs/EQ UCT Sonar PCB Manufacture_BOM .xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27932"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jtaylor\Documents\Sonar\EQs\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86E48EE7-E215-4B8A-9B55-4EDE5152B6B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12375" activeTab="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="89772A1_BOM" sheetId="1" r:id="rId1"/>
@@ -23,12 +29,15 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="107">
   <si>
     <t>Reference</t>
   </si>
@@ -351,26 +360,25 @@
   <si>
     <t>Total price
 (USD)</t>
+  </si>
+  <si>
+    <t>接受(acc)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="7">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="176" formatCode="0.000000_ "/>
-    <numFmt numFmtId="177" formatCode="0.000_ "/>
-    <numFmt numFmtId="178" formatCode="0.00_ "/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <numFmts count="3">
+    <numFmt numFmtId="168" formatCode="0.000000_ "/>
+    <numFmt numFmtId="169" formatCode="0.000_ "/>
+    <numFmt numFmtId="170" formatCode="0.00_ "/>
   </numFmts>
-  <fonts count="27">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="宋体"/>
+      <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -385,7 +393,6 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="微软雅黑"/>
-      <charset val="0"/>
     </font>
     <font>
       <b/>
@@ -420,152 +427,8 @@
       <name val="微软雅黑"/>
       <charset val="134"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="39">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -608,194 +471,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="11">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -831,251 +508,9 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1089,7 +524,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1098,10 +533,10 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1116,7 +551,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1125,7 +560,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1149,7 +584,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1158,65 +593,24 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="177" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="178" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="49">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
-    <cellStyle name="货币" xfId="2" builtinId="4"/>
-    <cellStyle name="百分比" xfId="3" builtinId="5"/>
-    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
-    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
-    <cellStyle name="超链接" xfId="6" builtinId="8"/>
-    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
-    <cellStyle name="注释" xfId="8" builtinId="10"/>
-    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
-    <cellStyle name="标题" xfId="10" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
-    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="输入" xfId="16" builtinId="20"/>
-    <cellStyle name="输出" xfId="17" builtinId="21"/>
-    <cellStyle name="计算" xfId="18" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
-    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
-    <cellStyle name="汇总" xfId="21" builtinId="25"/>
-    <cellStyle name="好" xfId="22" builtinId="26"/>
-    <cellStyle name="差" xfId="23" builtinId="27"/>
-    <cellStyle name="适中" xfId="24" builtinId="28"/>
-    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
-    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
-    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
-    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
-    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="23">
+  <dxfs count="34">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C6500"/>
@@ -1229,11 +623,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <color rgb="FF9C6500"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1248,13 +642,6 @@
       </fill>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <font>
         <color rgb="FF9C6500"/>
       </font>
@@ -1265,43 +652,270 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color rgb="FF9C6500"/>
+      </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFFFFF00"/>
+          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color rgb="FF9C6500"/>
+      </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
+          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <color rgb="FF9C6500"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C6500"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C6500"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C6500"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
         <color theme="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
         <color theme="1"/>
       </font>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <border>
+        <top style="thin">
+          <color theme="4"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
         <color theme="1"/>
       </font>
       <border>
@@ -1312,7 +926,7 @@
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
         <color theme="0"/>
       </font>
       <fill>
@@ -1340,160 +954,46 @@
           <color theme="4"/>
         </bottom>
         <horizontal style="thin">
-          <color theme="4" tint="0.399975585192419"/>
+          <color theme="4" tint="0.39994506668294322"/>
         </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <border>
-        <top style="thin">
-          <color theme="4"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
       </border>
     </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
     <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
-      <tableStyleElement type="wholeTable" dxfId="12"/>
-      <tableStyleElement type="headerRow" dxfId="11"/>
-      <tableStyleElement type="totalRow" dxfId="10"/>
-      <tableStyleElement type="firstColumn" dxfId="9"/>
-      <tableStyleElement type="lastColumn" dxfId="8"/>
-      <tableStyleElement type="firstRowStripe" dxfId="7"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="6"/>
+      <tableStyleElement type="wholeTable" dxfId="33"/>
+      <tableStyleElement type="headerRow" dxfId="32"/>
+      <tableStyleElement type="totalRow" dxfId="31"/>
+      <tableStyleElement type="firstColumn" dxfId="30"/>
+      <tableStyleElement type="lastColumn" dxfId="29"/>
+      <tableStyleElement type="firstRowStripe" dxfId="28"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="27"/>
     </tableStyle>
     <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
-      <tableStyleElement type="headerRow" dxfId="22"/>
-      <tableStyleElement type="totalRow" dxfId="21"/>
-      <tableStyleElement type="firstRowStripe" dxfId="20"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="19"/>
-      <tableStyleElement type="firstSubtotalRow" dxfId="18"/>
-      <tableStyleElement type="secondSubtotalRow" dxfId="17"/>
-      <tableStyleElement type="firstRowSubheading" dxfId="16"/>
-      <tableStyleElement type="secondRowSubheading" dxfId="15"/>
-      <tableStyleElement type="pageFieldLabels" dxfId="14"/>
-      <tableStyleElement type="pageFieldValues" dxfId="13"/>
+      <tableStyleElement type="headerRow" dxfId="26"/>
+      <tableStyleElement type="totalRow" dxfId="25"/>
+      <tableStyleElement type="firstRowStripe" dxfId="24"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="23"/>
+      <tableStyleElement type="firstSubtotalRow" dxfId="22"/>
+      <tableStyleElement type="secondSubtotalRow" dxfId="21"/>
+      <tableStyleElement type="firstRowSubheading" dxfId="20"/>
+      <tableStyleElement type="secondRowSubheading" dxfId="19"/>
+      <tableStyleElement type="pageFieldLabels" dxfId="18"/>
+      <tableStyleElement type="pageFieldValues" dxfId="17"/>
     </tableStyle>
   </tableStyles>
   <colors>
     <mruColors>
-      <color rgb="00FF0000"/>
-      <color rgb="00FFFF00"/>
+      <color rgb="FFFF0000"/>
+      <color rgb="FFFFFF00"/>
     </mruColors>
   </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1751,14 +1251,14 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E21"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
@@ -2119,36 +1619,34 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Q22"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="1" width="9" style="2"/>
-    <col min="2" max="2" width="21.875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="21.85546875" style="2" customWidth="1"/>
     <col min="3" max="3" width="9" style="2" customWidth="1"/>
-    <col min="4" max="4" width="23.7583333333333" style="2" customWidth="1"/>
+    <col min="4" max="4" width="23.7109375" style="2" customWidth="1"/>
     <col min="5" max="5" width="25" style="2" customWidth="1"/>
-    <col min="6" max="6" width="26.375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="26.42578125" style="2" customWidth="1"/>
     <col min="7" max="7" width="9" style="2"/>
-    <col min="8" max="8" width="13.5" style="3" customWidth="1"/>
-    <col min="9" max="9" width="14.5" style="3" customWidth="1"/>
+    <col min="8" max="8" width="13.42578125" style="3" customWidth="1"/>
+    <col min="9" max="9" width="14.42578125" style="3" customWidth="1"/>
     <col min="10" max="11" width="9" style="2"/>
-    <col min="12" max="12" width="21.7583333333333" style="2" customWidth="1"/>
-    <col min="13" max="13" width="22.2583333333333" style="2" customWidth="1"/>
-    <col min="14" max="14" width="34.5" style="2" customWidth="1"/>
-    <col min="15" max="15" width="19.375" style="2" customWidth="1"/>
-    <col min="16" max="16" width="32.125" style="2" customWidth="1"/>
-    <col min="17" max="17" width="18.125" style="2" customWidth="1"/>
+    <col min="12" max="12" width="21.7109375" style="2" customWidth="1"/>
+    <col min="13" max="13" width="22.28515625" style="2" customWidth="1"/>
+    <col min="14" max="14" width="34.42578125" style="2" customWidth="1"/>
+    <col min="15" max="15" width="19.42578125" style="2" customWidth="1"/>
+    <col min="16" max="16" width="32.140625" style="2" customWidth="1"/>
+    <col min="17" max="17" width="18.140625" style="2" customWidth="1"/>
     <col min="18" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="33" spans="1:17">
+    <row r="1" spans="1:17" ht="33">
       <c r="B1" s="4" t="s">
         <v>0</v>
       </c>
@@ -2222,11 +1720,11 @@
         <v>50</v>
       </c>
       <c r="H2" s="12">
-        <v>0.117056</v>
+        <v>0.11705599999999999</v>
       </c>
       <c r="I2" s="12">
         <f>C2*H2</f>
-        <v>0.234112</v>
+        <v>0.23411199999999999</v>
       </c>
       <c r="J2" s="13">
         <v>380</v>
@@ -2247,7 +1745,9 @@
         <v>81</v>
       </c>
       <c r="P2" s="4"/>
-      <c r="Q2" s="14"/>
+      <c r="Q2" s="14" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="3" spans="1:17">
       <c r="A3" s="4">
@@ -2273,11 +1773,11 @@
         <v>50</v>
       </c>
       <c r="H3" s="15">
-        <v>0.0178994117647059</v>
+        <v>1.78994117647059E-2</v>
       </c>
       <c r="I3" s="12">
         <f t="shared" ref="I3:I21" si="1">C3*H3</f>
-        <v>0.0357988235294118</v>
+        <v>3.57988235294118E-2</v>
       </c>
       <c r="J3" s="4" t="s">
         <v>82</v>
@@ -2298,7 +1798,9 @@
         <v>81</v>
       </c>
       <c r="P3" s="4"/>
-      <c r="Q3" s="14"/>
+      <c r="Q3" s="14" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="4" spans="1:17">
       <c r="A4" s="4">
@@ -2324,11 +1826,11 @@
         <v>75</v>
       </c>
       <c r="H4" s="15">
-        <v>0.0653572058823529</v>
+        <v>6.5357205882352901E-2</v>
       </c>
       <c r="I4" s="12">
         <f t="shared" si="1"/>
-        <v>0.196071617647059</v>
+        <v>0.19607161764705899</v>
       </c>
       <c r="J4" s="16">
         <v>30150</v>
@@ -2349,9 +1851,11 @@
         <v>85</v>
       </c>
       <c r="P4" s="17"/>
-      <c r="Q4" s="14"/>
-    </row>
-    <row r="5" ht="33" spans="1:17">
+      <c r="Q4" s="14" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" ht="33">
       <c r="A5" s="4">
         <v>4</v>
       </c>
@@ -2375,11 +1879,11 @@
         <v>425</v>
       </c>
       <c r="H5" s="12">
-        <v>0.0262605882352941</v>
+        <v>2.6260588235294102E-2</v>
       </c>
       <c r="I5" s="12">
         <f t="shared" si="1"/>
-        <v>0.44643</v>
+        <v>0.44642999999999999</v>
       </c>
       <c r="J5" s="18" t="s">
         <v>86</v>
@@ -2398,9 +1902,11 @@
       </c>
       <c r="O5" s="17"/>
       <c r="P5" s="17"/>
-      <c r="Q5" s="14"/>
-    </row>
-    <row r="6" ht="115.5" spans="1:17">
+      <c r="Q5" s="14" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" ht="132">
       <c r="A6" s="4">
         <v>5</v>
       </c>
@@ -2424,11 +1930,11 @@
         <v>1000</v>
       </c>
       <c r="H6" s="15">
-        <v>0.124293352941176</v>
+        <v>0.12429335294117599</v>
       </c>
       <c r="I6" s="12">
         <f t="shared" si="1"/>
-        <v>4.97173411764706</v>
+        <v>4.9717341176470597</v>
       </c>
       <c r="J6" s="16">
         <v>37573</v>
@@ -2449,7 +1955,9 @@
         <v>81</v>
       </c>
       <c r="P6" s="17"/>
-      <c r="Q6" s="14"/>
+      <c r="Q6" s="14" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="7" spans="1:17">
       <c r="A7" s="4">
@@ -2475,11 +1983,11 @@
         <v>250</v>
       </c>
       <c r="H7" s="15">
-        <v>0.504511764705882</v>
+        <v>0.50451176470588199</v>
       </c>
       <c r="I7" s="12">
         <f t="shared" si="1"/>
-        <v>5.04511764705882</v>
+        <v>5.0451176470588202</v>
       </c>
       <c r="J7" s="4">
         <v>866</v>
@@ -2500,7 +2008,9 @@
         <v>85</v>
       </c>
       <c r="P7" s="17"/>
-      <c r="Q7" s="14"/>
+      <c r="Q7" s="14" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="8" spans="1:17">
       <c r="A8" s="4">
@@ -2526,11 +2036,11 @@
         <v>25</v>
       </c>
       <c r="H8" s="15">
-        <v>7.21013117647059</v>
+        <v>7.2101311764705898</v>
       </c>
       <c r="I8" s="12">
         <f t="shared" si="1"/>
-        <v>7.21013117647059</v>
+        <v>7.2101311764705898</v>
       </c>
       <c r="J8" s="4">
         <v>161</v>
@@ -2551,7 +2061,9 @@
         <v>85</v>
       </c>
       <c r="P8" s="17"/>
-      <c r="Q8" s="14"/>
+      <c r="Q8" s="14" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="9" spans="1:17">
       <c r="A9" s="4">
@@ -2577,11 +2089,11 @@
         <v>25</v>
       </c>
       <c r="H9" s="15">
-        <v>3.94436470588235</v>
+        <v>3.9443647058823501</v>
       </c>
       <c r="I9" s="12">
         <f t="shared" si="1"/>
-        <v>3.94436470588235</v>
+        <v>3.9443647058823501</v>
       </c>
       <c r="J9" s="16">
         <v>3936</v>
@@ -2602,7 +2114,9 @@
         <v>85</v>
       </c>
       <c r="P9" s="17"/>
-      <c r="Q9" s="14"/>
+      <c r="Q9" s="14" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="10" spans="1:17">
       <c r="A10" s="4">
@@ -2628,7 +2142,7 @@
         <v>475</v>
       </c>
       <c r="H10" s="15">
-        <v>0.0687970588235294</v>
+        <v>6.8797058823529406E-2</v>
       </c>
       <c r="I10" s="12">
         <f t="shared" si="1"/>
@@ -2653,7 +2167,9 @@
         <v>85</v>
       </c>
       <c r="P10" s="17"/>
-      <c r="Q10" s="14"/>
+      <c r="Q10" s="14" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="11" spans="1:17">
       <c r="A11" s="4">
@@ -2679,11 +2195,11 @@
         <v>50</v>
       </c>
       <c r="H11" s="15">
-        <v>0.0974625</v>
+        <v>9.7462499999999994E-2</v>
       </c>
       <c r="I11" s="12">
         <f t="shared" si="1"/>
-        <v>0.194925</v>
+        <v>0.19492499999999999</v>
       </c>
       <c r="J11" s="16">
         <v>11187</v>
@@ -2704,7 +2220,9 @@
         <v>85</v>
       </c>
       <c r="P11" s="17"/>
-      <c r="Q11" s="14"/>
+      <c r="Q11" s="14" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="12" spans="1:17">
       <c r="A12" s="4">
@@ -2730,7 +2248,7 @@
         <v>400</v>
       </c>
       <c r="H12" s="12">
-        <v>0.0687970588235294</v>
+        <v>6.8797058823529406E-2</v>
       </c>
       <c r="I12" s="12">
         <f t="shared" si="1"/>
@@ -2755,9 +2273,11 @@
         <v>85</v>
       </c>
       <c r="P12" s="17"/>
-      <c r="Q12" s="14"/>
-    </row>
-    <row r="13" ht="33" spans="1:17">
+      <c r="Q12" s="14" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" ht="49.5">
       <c r="A13" s="4">
         <v>12</v>
       </c>
@@ -2781,7 +2301,7 @@
         <v>425</v>
       </c>
       <c r="H13" s="15">
-        <v>0.0905827941176471</v>
+        <v>9.0582794117647095E-2</v>
       </c>
       <c r="I13" s="12">
         <f t="shared" si="1"/>
@@ -2808,7 +2328,9 @@
       <c r="P13" s="20" t="s">
         <v>98</v>
       </c>
-      <c r="Q13" s="14"/>
+      <c r="Q13" s="14" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="14" spans="1:17">
       <c r="A14" s="4">
@@ -2834,7 +2356,7 @@
         <v>400</v>
       </c>
       <c r="H14" s="15">
-        <v>0.0687970588235294</v>
+        <v>6.8797058823529406E-2</v>
       </c>
       <c r="I14" s="12">
         <f t="shared" si="1"/>
@@ -2859,7 +2381,9 @@
         <v>85</v>
       </c>
       <c r="P14" s="17"/>
-      <c r="Q14" s="14"/>
+      <c r="Q14" s="14" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="15" spans="1:17">
       <c r="A15" s="4">
@@ -2885,7 +2409,7 @@
         <v>1200</v>
       </c>
       <c r="H15" s="15">
-        <v>0.0536617058823529</v>
+        <v>5.3661705882352903E-2</v>
       </c>
       <c r="I15" s="12">
         <f t="shared" si="1"/>
@@ -2910,7 +2434,9 @@
         <v>85</v>
       </c>
       <c r="P15" s="17"/>
-      <c r="Q15" s="14"/>
+      <c r="Q15" s="14" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="16" spans="1:17">
       <c r="A16" s="4">
@@ -2936,11 +2462,11 @@
         <v>75</v>
       </c>
       <c r="H16" s="15">
-        <v>0.418058823529412</v>
+        <v>0.41805882352941198</v>
       </c>
       <c r="I16" s="12">
         <f t="shared" si="1"/>
-        <v>1.25417647058824</v>
+        <v>1.2541764705882401</v>
       </c>
       <c r="J16" s="4">
         <v>1971</v>
@@ -2961,7 +2487,9 @@
         <v>81</v>
       </c>
       <c r="P16" s="17"/>
-      <c r="Q16" s="14"/>
+      <c r="Q16" s="14" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="17" spans="1:17">
       <c r="A17" s="4">
@@ -2987,11 +2515,11 @@
         <v>25</v>
       </c>
       <c r="H17" s="12">
-        <v>0.554029411764706</v>
+        <v>0.55402941176470599</v>
       </c>
       <c r="I17" s="12">
         <f t="shared" si="1"/>
-        <v>0.554029411764706</v>
+        <v>0.55402941176470599</v>
       </c>
       <c r="J17" s="18">
         <v>4232</v>
@@ -3012,7 +2540,9 @@
         <v>81</v>
       </c>
       <c r="P17" s="17"/>
-      <c r="Q17" s="14"/>
+      <c r="Q17" s="14" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="18" spans="1:17">
       <c r="A18" s="4">
@@ -3042,7 +2572,7 @@
       </c>
       <c r="I18" s="12">
         <f t="shared" si="1"/>
-        <v>2.61658147058823</v>
+        <v>2.6165814705882302</v>
       </c>
       <c r="J18" s="16">
         <v>120019</v>
@@ -3063,7 +2593,9 @@
         <v>85</v>
       </c>
       <c r="P18" s="17"/>
-      <c r="Q18" s="14"/>
+      <c r="Q18" s="14" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="19" spans="1:17">
       <c r="A19" s="4">
@@ -3089,11 +2621,11 @@
         <v>25</v>
       </c>
       <c r="H19" s="15">
-        <v>0.623029411764706</v>
+        <v>0.62302941176470605</v>
       </c>
       <c r="I19" s="12">
         <f t="shared" si="1"/>
-        <v>0.623029411764706</v>
+        <v>0.62302941176470605</v>
       </c>
       <c r="J19" s="4">
         <v>996</v>
@@ -3114,9 +2646,11 @@
         <v>81</v>
       </c>
       <c r="P19" s="4"/>
-      <c r="Q19" s="14"/>
-    </row>
-    <row r="20" s="1" customFormat="1" spans="1:17">
+      <c r="Q19" s="14" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" s="1" customFormat="1">
       <c r="A20" s="4">
         <v>19</v>
       </c>
@@ -3140,11 +2674,11 @@
         <v>50</v>
       </c>
       <c r="H20" s="23">
-        <v>38.2850470588235</v>
+        <v>38.285047058823501</v>
       </c>
       <c r="I20" s="12">
         <f t="shared" si="1"/>
-        <v>76.5700941176471</v>
+        <v>76.570094117647102</v>
       </c>
       <c r="J20" s="22">
         <v>315</v>
@@ -3165,9 +2699,11 @@
         <v>85</v>
       </c>
       <c r="P20" s="24"/>
-      <c r="Q20" s="14"/>
-    </row>
-    <row r="21" s="1" customFormat="1" ht="33" spans="1:17">
+      <c r="Q20" s="14" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" s="1" customFormat="1" ht="49.5">
       <c r="A21" s="4">
         <v>20</v>
       </c>
@@ -3191,7 +2727,7 @@
         <v>100</v>
       </c>
       <c r="H21" s="23">
-        <v>2.99541176470588</v>
+        <v>2.9954117647058802</v>
       </c>
       <c r="I21" s="12">
         <f t="shared" si="1"/>
@@ -3216,9 +2752,11 @@
       <c r="P21" s="25" t="s">
         <v>104</v>
       </c>
-      <c r="Q21" s="14"/>
-    </row>
-    <row r="22" ht="35" customHeight="1" spans="1:17">
+      <c r="Q21" s="14" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" ht="35.1" customHeight="1">
       <c r="A22" s="4">
         <v>21</v>
       </c>
@@ -3232,50 +2770,49 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="L1">
-    <cfRule type="duplicateValues" dxfId="0" priority="14"/>
-    <cfRule type="duplicateValues" dxfId="1" priority="15"/>
-    <cfRule type="duplicateValues" dxfId="2" priority="16"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="M1">
-    <cfRule type="duplicateValues" dxfId="2" priority="11"/>
-    <cfRule type="timePeriod" dxfId="4" priority="12" timePeriod="yesterday">
+    <cfRule type="duplicateValues" dxfId="12" priority="11"/>
+    <cfRule type="timePeriod" dxfId="11" priority="12" timePeriod="yesterday">
       <formula>FLOOR(M1,1)=TODAY()-1</formula>
     </cfRule>
-    <cfRule type="duplicateValues" dxfId="0" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1">
-    <cfRule type="duplicateValues" dxfId="2" priority="8"/>
-    <cfRule type="timePeriod" dxfId="4" priority="9" timePeriod="yesterday">
+    <cfRule type="duplicateValues" dxfId="9" priority="8"/>
+    <cfRule type="timePeriod" dxfId="8" priority="9" timePeriod="yesterday">
       <formula>FLOOR(N1,1)=TODAY()-1</formula>
     </cfRule>
-    <cfRule type="duplicateValues" dxfId="0" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="O1">
-    <cfRule type="duplicateValues" dxfId="2" priority="5"/>
-    <cfRule type="timePeriod" dxfId="4" priority="6" timePeriod="yesterday">
+    <cfRule type="duplicateValues" dxfId="6" priority="5"/>
+    <cfRule type="timePeriod" dxfId="5" priority="6" timePeriod="yesterday">
       <formula>FLOOR(O1,1)=TODAY()-1</formula>
     </cfRule>
-    <cfRule type="duplicateValues" dxfId="0" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q1">
-    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
-    <cfRule type="timePeriod" dxfId="4" priority="3" timePeriod="yesterday">
+    <cfRule type="duplicateValues" dxfId="3" priority="2"/>
+    <cfRule type="timePeriod" dxfId="2" priority="3" timePeriod="yesterday">
       <formula>FLOOR(Q1,1)=TODAY()-1</formula>
     </cfRule>
-    <cfRule type="duplicateValues" dxfId="0" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q2:Q21">
-    <cfRule type="expression" dxfId="5" priority="1">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>OR(MID($B2,2,1)="-",MID($B2,3,1)="-")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q2:Q21">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q2:Q21" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"接受(acc),拒绝(rej)"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>